<commit_message>
Update full vocab exercise identifiers
</commit_message>
<xml_diff>
--- a/docs/assets/3rdparty/source/VocExcel-ice-cream-flavor-collections.xlsx
+++ b/docs/assets/3rdparty/source/VocExcel-ice-cream-flavor-collections.xlsx
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="410">
   <si>
     <t>Version:</t>
   </si>
@@ -1705,7 +1705,7 @@
     <t>FRUIT FLAVORS</t>
   </si>
   <si>
-    <t>icf:45b0a9d3-d3c9-4c19-b4ef-0511a8827101</t>
+    <t>icf:2</t>
   </si>
   <si>
     <t>Banana</t>
@@ -1714,7 +1714,7 @@
     <t>Banana ice cream flavor</t>
   </si>
   <si>
-    <t>icf:abf359ff-5c42-42e1-91a5-21973879f6f0</t>
+    <t>icf:3</t>
   </si>
   <si>
     <t>Black raspberry</t>
@@ -1723,7 +1723,7 @@
     <t>Black raspberry ice cream flavor</t>
   </si>
   <si>
-    <t>icf:0f748e6f-ae0b-49a9-bac9-98db1de6fd04</t>
+    <t>icf:4</t>
   </si>
   <si>
     <t xml:space="preserve">Cherry </t>
@@ -1735,7 +1735,7 @@
     <t>Amaretto cherry, black cherry</t>
   </si>
   <si>
-    <t>icf:bf94fff7-9ef5-4af6-91dc-bf332e1bbd72</t>
+    <t>icf:5</t>
   </si>
   <si>
     <t>Cinnamon apple</t>
@@ -1744,7 +1744,7 @@
     <t>Cinnamon apple ice cream flavor</t>
   </si>
   <si>
-    <t>icf:556b0f61-f107-4519-8bbe-cf3c29d840bb</t>
+    <t>icf:6</t>
   </si>
   <si>
     <t>Grape</t>
@@ -1753,7 +1753,7 @@
     <t>Grape ice cream flavor</t>
   </si>
   <si>
-    <t>icf:79aaa965-5e88-4a01-8b5a-87438ff46cf6</t>
+    <t>icf:7</t>
   </si>
   <si>
     <t xml:space="preserve">Lúcuma </t>
@@ -1762,13 +1762,13 @@
     <t xml:space="preserve"> A popular Peruvian ice cream flavor with an orange color and a sweet nutty taste</t>
   </si>
   <si>
-    <t>icf:4343af06-9db2-43d4-920a-61d349ef42f5</t>
+    <t>icf:8</t>
   </si>
   <si>
     <t>Mamey</t>
   </si>
   <si>
-    <t>icf:f476202a-b952-4b55-8877-33570ee26cf5</t>
+    <t>icf:9</t>
   </si>
   <si>
     <t>Mango</t>
@@ -1777,7 +1777,7 @@
     <t>Mango ice cream flavor</t>
   </si>
   <si>
-    <t>icf:cd2071b4-cb2e-4c12-ad82-fa7b2c844899</t>
+    <t>icf:10</t>
   </si>
   <si>
     <t xml:space="preserve">Moon mist </t>
@@ -1786,7 +1786,7 @@
     <t>A blend of grape, banana, and blue raspberry (or sometimes bubblegum) flavors, popular in Atlantic Canada. The flavors are generally blended together to give a mist-like texture.</t>
   </si>
   <si>
-    <t>icf:61ed4c66-f7d8-40c9-8866-cc4bdee3ea44</t>
+    <t>icf:11</t>
   </si>
   <si>
     <t>Passion fruit</t>
@@ -1795,7 +1795,7 @@
     <t>Passion fruit ice cream flavor</t>
   </si>
   <si>
-    <t>icf:9e8afe4c-f6db-40e3-a625-7dbeadc1a3d5</t>
+    <t>icf:12</t>
   </si>
   <si>
     <t>Pumpkin</t>
@@ -1804,7 +1804,7 @@
     <t>Pumpkin ice cream flavor</t>
   </si>
   <si>
-    <t>icf:a5120bb8-2a39-4b7e-95e4-c05646ab53e2</t>
+    <t>icf:13</t>
   </si>
   <si>
     <t xml:space="preserve">Raspberry ripple </t>
@@ -1813,7 +1813,7 @@
     <t xml:space="preserve"> Consists of raspberry syrup injected into vanilla ice cream.</t>
   </si>
   <si>
-    <t>icf:7b276e8c-ac83-4eb0-8b8d-e26f0f00d190</t>
+    <t>icf:14</t>
   </si>
   <si>
     <t>Rum raisin</t>
@@ -1822,7 +1822,7 @@
     <t>Rum raisin ice cream flavor</t>
   </si>
   <si>
-    <t>icf:ccb7b867-4f44-4eea-bd09-99f964664733</t>
+    <t>icf:15</t>
   </si>
   <si>
     <t>Strawberry</t>
@@ -1831,7 +1831,7 @@
     <t>Strawberry ice cream flavor</t>
   </si>
   <si>
-    <t>icf:b8af11ac-39c5-4547-8ff0-1cb77e50f9d5</t>
+    <t>icf:16</t>
   </si>
   <si>
     <t>Strawberry cheesecake</t>
@@ -1840,7 +1840,7 @@
     <t>Strawberry cheesecake ice cream flavor</t>
   </si>
   <si>
-    <t>icf:bd9289fa-9715-4a2e-89bd-bc4f705dc167</t>
+    <t>icf:17</t>
   </si>
   <si>
     <t>Superman</t>
@@ -1849,7 +1849,7 @@
     <t xml:space="preserve">Superman ice cream is a three-flavor ice cream that usually appears in red, blue, and yellow. </t>
   </si>
   <si>
-    <t>icf:0e9b17d8-339c-4a55-8157-03b15be56f76</t>
+    <t>icf:18</t>
   </si>
   <si>
     <t>Teaberry</t>
@@ -1858,7 +1858,7 @@
     <t>Teaberry ice cream is an ice cream flavor made with the eastern teaberry fruit. </t>
   </si>
   <si>
-    <t>icf:d35b1641-f112-4ab5-83fe-95e98229f4e7</t>
+    <t>icf:19</t>
   </si>
   <si>
     <t xml:space="preserve">Tiger tail </t>
@@ -1867,7 +1867,7 @@
     <t>A flavor popular in Canada, consisting of orange-flavored ice cream with swirls of black licorice</t>
   </si>
   <si>
-    <t>icf:a1a144fd-3f41-4961-9bb1-47ac783232b5</t>
+    <t>icf:20</t>
   </si>
   <si>
     <t>Tutti frutti</t>
@@ -1876,7 +1876,7 @@
     <t>Tutti frutti ice cream flavor</t>
   </si>
   <si>
-    <t>icf:9de1e781-4733-4cbe-8cb2-143d7a4ed92f</t>
+    <t>icf:21</t>
   </si>
   <si>
     <t>Watermelon</t>
@@ -1885,7 +1885,7 @@
     <t>CHOCOLATE, NUTS AND OTHER SWEETS</t>
   </si>
   <si>
-    <t>icf:e702da60-1dbe-48ee-891f-e1de99ee07d5</t>
+    <t>icf:23</t>
   </si>
   <si>
     <t xml:space="preserve">Biscuit Tortoni </t>
@@ -1894,7 +1894,7 @@
     <t>An ice cream made with eggs and heavy cream, often containing chopped cherries or topped with minced almonds or crumbled macaroons</t>
   </si>
   <si>
-    <t>icf:2f524245-e21c-4c02-966d-f3b4022535ea</t>
+    <t>icf:24</t>
   </si>
   <si>
     <t xml:space="preserve">Blue moon </t>
@@ -1903,7 +1903,7 @@
     <t>An ice cream flavor with bright blue coloring, available in the Upper Midwest of the United States</t>
   </si>
   <si>
-    <t>icf:c4c2344c-4b1b-462a-b9f9-e1b03faeb0dd</t>
+    <t>icf:25</t>
   </si>
   <si>
     <t>Bubblegum</t>
@@ -1912,7 +1912,7 @@
     <t>Bubblegum ice cream flavor</t>
   </si>
   <si>
-    <t>icf:f4fe093d-96d6-4419-8079-1fdba8a479cc</t>
+    <t>icf:26</t>
   </si>
   <si>
     <t xml:space="preserve">Butter Brickle </t>
@@ -1921,7 +1921,7 @@
     <t>The registered trademark of a toffee ice cream flavoring and of a toffee-centered chocolate-covered candy bar similar to the Heath bar, introduced by the Blackstone Hotel in Omaha, Nebraska, in the 1920s. Alternately, it is often prepared and sold as butter vanilla-flavored ice cream with tiny flecks of butter toffee instead of chunks of Heath bar.</t>
   </si>
   <si>
-    <t>icf:66dcdd54-fffb-4d29-90bc-0be9a9d052b5</t>
+    <t>icf:27</t>
   </si>
   <si>
     <t>Butterscotch</t>
@@ -1930,7 +1930,7 @@
     <t>Butterscotch ice cream flavor</t>
   </si>
   <si>
-    <t>icf:a61185c1-786a-4a93-8964-0d53686baddd</t>
+    <t>icf:28</t>
   </si>
   <si>
     <t xml:space="preserve">Butter pecan </t>
@@ -1939,7 +1939,7 @@
     <t>A smooth vanilla ice cream with a slight buttery flavor, with pecans added.</t>
   </si>
   <si>
-    <t>icf:aa64a8c2-8dbb-428b-94f9-fc328870d3ec</t>
+    <t>icf:29</t>
   </si>
   <si>
     <t>Cake batter</t>
@@ -1948,7 +1948,7 @@
     <t>Cake batter ice cream flavor</t>
   </si>
   <si>
-    <t>icf:2307a8fb-e802-403a-b255-6ec1a57677aa</t>
+    <t>icf:30</t>
   </si>
   <si>
     <t>Caramel</t>
@@ -1957,7 +1957,7 @@
     <t>Caramel ice cream flavor</t>
   </si>
   <si>
-    <t>icf:e8555003-5203-47d4-af04-70798add66ad</t>
+    <t>icf:31</t>
   </si>
   <si>
     <t>Chocolate</t>
@@ -1966,7 +1966,7 @@
     <t>Chocolate ice cream is ice cream with natural or artificial chocolate flavoring.</t>
   </si>
   <si>
-    <t>icf:f7bbc944-ecdc-4517-8f71-6ac6653db5c4</t>
+    <t>icf:32</t>
   </si>
   <si>
     <t xml:space="preserve">Chocolate chip </t>
@@ -1975,7 +1975,7 @@
     <t>Vanilla base, with chunks of solid chocolate. Declining in popularity in the 2020s. Sometimes chocolate ice cream was used, which was usually called "Chocolate chocolate chip"</t>
   </si>
   <si>
-    <t>icf:678299ea-ae67-4736-b109-02f3b5c2e752</t>
+    <t>icf:33</t>
   </si>
   <si>
     <t>Chocolate chip cookie dough</t>
@@ -1984,7 +1984,7 @@
     <t>Chocolate chip cookie dough ice cream flavor</t>
   </si>
   <si>
-    <t>icf:cd7ecf43-79b3-4495-98a5-fea33b86a29c</t>
+    <t>icf:34</t>
   </si>
   <si>
     <t>Coffee</t>
@@ -1993,7 +1993,7 @@
     <t>Coffee ice cream is an ice cream flavor made with coffee or coffee flavoring.</t>
   </si>
   <si>
-    <t>icf:10cdc74f-c236-42cf-bb32-33f40c882189</t>
+    <t>icf:35</t>
   </si>
   <si>
     <t>Cookies and cream</t>
@@ -2002,7 +2002,7 @@
     <t>Cookies and cream ice cream flavor</t>
   </si>
   <si>
-    <t>icf:1619cc1c-c75b-45d1-bdaf-ced29978673f</t>
+    <t>icf:36</t>
   </si>
   <si>
     <t>Cotton candy</t>
@@ -2011,7 +2011,7 @@
     <t>Cotton candy ice cream flavor</t>
   </si>
   <si>
-    <t>icf:bbe41b1a-5eb1-4d35-af25-673b0c0c842d</t>
+    <t>icf:37</t>
   </si>
   <si>
     <t>Dulce de leche</t>
@@ -2020,7 +2020,7 @@
     <t>Dulce de leche ice cream flavor</t>
   </si>
   <si>
-    <t>icf:98656441-5fd4-42e8-bd11-cfce8fae4a86</t>
+    <t>icf:38</t>
   </si>
   <si>
     <t>Earl Grey tea</t>
@@ -2029,7 +2029,7 @@
     <t>Earl Grey tea ice cream flavor</t>
   </si>
   <si>
-    <t>icf:6148a62f-1ae4-4797-9f6a-359f17c2c60a</t>
+    <t>icf:39</t>
   </si>
   <si>
     <t>Eggnog</t>
@@ -2038,7 +2038,7 @@
     <t>Eggnog ice cream flavor</t>
   </si>
   <si>
-    <t>icf:f8892819-70b5-4efc-8e42-43d1024d943e</t>
+    <t>icf:40</t>
   </si>
   <si>
     <t>French vanilla</t>
@@ -2047,7 +2047,7 @@
     <t>French vanilla ice cream flavor</t>
   </si>
   <si>
-    <t>icf:d4ef5ab1-2fd4-4b70-b7a0-ad79605f5e4e</t>
+    <t>icf:41</t>
   </si>
   <si>
     <t xml:space="preserve">Goody Goody Gum Drops </t>
@@ -2056,7 +2056,7 @@
     <t>Goody Goody Gum Drops ice cream flavor, unique to New Zealand</t>
   </si>
   <si>
-    <t>icf:5c2bad30-3036-4394-abef-1daf0cb6351d</t>
+    <t>icf:42</t>
   </si>
   <si>
     <t>Green tea</t>
@@ -2065,7 +2065,7 @@
     <t>Green tea  ice cream flavor</t>
   </si>
   <si>
-    <t>icf:07ff3c57-c075-4a95-be6a-99955621dd5c</t>
+    <t>icf:43</t>
   </si>
   <si>
     <t>Halva</t>
@@ -2074,7 +2074,7 @@
     <t>Halva ice cream flavor</t>
   </si>
   <si>
-    <t>icf:3c71c026-00b2-435e-bb8b-66d006e7b133</t>
+    <t>icf:44</t>
   </si>
   <si>
     <t xml:space="preserve">Hokey pokey </t>
@@ -2083,7 +2083,7 @@
     <t>a flavor of ice cream in New Zealand, consisting of plain vanilla ice cream with small, solid lumps of honeycomb toffee</t>
   </si>
   <si>
-    <t>icf:ade1b5f0-58c6-46a8-8faa-6ed4224c72b7</t>
+    <t>icf:45</t>
   </si>
   <si>
     <t>Maple</t>
@@ -2092,7 +2092,7 @@
     <t>Maple ice cream flavor</t>
   </si>
   <si>
-    <t>icf:23798250-a926-42ba-95ce-c5576efa0bec</t>
+    <t>icf:46</t>
   </si>
   <si>
     <t xml:space="preserve">Mint chocolate chip </t>
@@ -2101,7 +2101,7 @@
     <t>Composed of mint ice cream with small chocolate chips. In some cases the liqueur crème de menthe is used to provide the mint flavor, but in most cases peppermint or spearmint flavoring is used.</t>
   </si>
   <si>
-    <t>icf:a886dea1-e597-40a2-84c2-f91f1750c724</t>
+    <t>icf:47</t>
   </si>
   <si>
     <t>Moose tracks</t>
@@ -2110,7 +2110,7 @@
     <t>Moose tracks ice cream flavor</t>
   </si>
   <si>
-    <t>icf:06f52b88-9ad0-4214-bf41-f5c23514d2cd</t>
+    <t>icf:48</t>
   </si>
   <si>
     <t xml:space="preserve">Neapolitan </t>
@@ -2119,7 +2119,7 @@
     <t xml:space="preserve"> Composed of vanilla, chocolate and strawberry ice cream together side by side</t>
   </si>
   <si>
-    <t>icf:28d8e6bb-6003-451e-b21e-292b4c5067f4</t>
+    <t>icf:49</t>
   </si>
   <si>
     <t>Pistachio</t>
@@ -2128,7 +2128,7 @@
     <t>Pistachio ice cream flavor</t>
   </si>
   <si>
-    <t>icf:48493fe1-dccb-45d0-9082-90ee9cb2e2f6</t>
+    <t>icf:50</t>
   </si>
   <si>
     <t>Peanut butter</t>
@@ -2137,7 +2137,7 @@
     <t>Peanut butter ice cream flavor</t>
   </si>
   <si>
-    <t>icf:cf5e8785-f0d9-4d8f-bcd8-c196b3751051</t>
+    <t>icf:51</t>
   </si>
   <si>
     <t xml:space="preserve">Rocky road </t>
@@ -2146,7 +2146,7 @@
     <t>Although there are variations from the original flavor, it is traditionally composed of chocolate ice cream, nuts, and whole or diced marshmallows, or sometimes replaced with marshmallow creme, a more fluid version</t>
   </si>
   <si>
-    <t>icf:a91c45b3-4168-4326-ba6f-6300858fde67</t>
+    <t>icf:52</t>
   </si>
   <si>
     <t>Rose</t>
@@ -2155,7 +2155,7 @@
     <t>Rose ice cream flavor</t>
   </si>
   <si>
-    <t>icf:a06e660a-7ca5-4213-88a9-5c2ea3574899</t>
+    <t>icf:53</t>
   </si>
   <si>
     <t xml:space="preserve">Spumoni </t>
@@ -2164,7 +2164,7 @@
     <t>A molded Italian ice cream made with layers of different colors and flavors, usually containing candied fruits and nuts.</t>
   </si>
   <si>
-    <t>icf:8f32f706-4827-4b52-8658-97af4cfa0398</t>
+    <t>icf:54</t>
   </si>
   <si>
     <t>Stracciatella</t>
@@ -2173,7 +2173,7 @@
     <t>Stracciatella ice cream flavor</t>
   </si>
   <si>
-    <t>icf:295b3fc1-a889-4960-bdbd-304392d1f0ec</t>
+    <t>icf:55</t>
   </si>
   <si>
     <t>Thai tea</t>
@@ -2182,7 +2182,7 @@
     <t>Thai tea ice cream flavor</t>
   </si>
   <si>
-    <t>icf:033da6cd-a916-467c-bbea-a6cd7b2fd9a3</t>
+    <t>icf:56</t>
   </si>
   <si>
     <t xml:space="preserve">Tramontana </t>
@@ -2191,7 +2191,7 @@
     <t>Composed of dark chocolate, white chocolate, dulce de leche and cookies.</t>
   </si>
   <si>
-    <t>icf:f8463b04-fa44-41b7-bb42-acc83a089cbb</t>
+    <t>icf:57</t>
   </si>
   <si>
     <t>Vanilla</t>
@@ -2203,7 +2203,7 @@
     <t>SAVORY FLAVORS</t>
   </si>
   <si>
-    <t>icf:cc6b3ba1-b7ef-4ea9-b60a-77c52c1bb74d</t>
+    <t>icf:59</t>
   </si>
   <si>
     <t xml:space="preserve">Bacon </t>
@@ -2212,7 +2212,7 @@
     <t>A modern invention, generally created by adding bacon to egg custard and freezing the mixture</t>
   </si>
   <si>
-    <t>icf:e54eea7d-074b-4d7b-8d73-d0df22b1f3e3</t>
+    <t>icf:60</t>
   </si>
   <si>
     <t>Beer</t>
@@ -2221,7 +2221,7 @@
     <t>Beer ice cream flavor</t>
   </si>
   <si>
-    <t>icf:2db0fe98-c26f-4cde-955e-53e0cbe5ee8e</t>
+    <t>icf:61</t>
   </si>
   <si>
     <t>Carrot</t>
@@ -2230,7 +2230,7 @@
     <t>Carrot ice cream flavor</t>
   </si>
   <si>
-    <t>icf:abb0e61b-5c54-4984-a13b-780563887653</t>
+    <t>icf:62</t>
   </si>
   <si>
     <t>Cheese</t>
@@ -2239,7 +2239,7 @@
     <t>Cheese ice cream flavor</t>
   </si>
   <si>
-    <t>icf:f550c468-b125-49ff-a3f2-1876954f7f73</t>
+    <t>icf:63</t>
   </si>
   <si>
     <t xml:space="preserve">Crab </t>
@@ -2248,7 +2248,7 @@
     <t>A Japanese creation,it is described as having a sweet taste; the island of Hokkaido, Japan, is known for manufacturing it</t>
   </si>
   <si>
-    <t>icf:1671e56f-52db-48af-a0a5-e45f8eb66053</t>
+    <t>icf:64</t>
   </si>
   <si>
     <t>Creole cream cheese</t>
@@ -2257,7 +2257,7 @@
     <t>Creole cream cheese ice cream flavor</t>
   </si>
   <si>
-    <t>icf:88947dcc-ef36-4bda-b26f-d91b9bbb92d9</t>
+    <t>icf:65</t>
   </si>
   <si>
     <t>Garlic</t>
@@ -2266,7 +2266,7 @@
     <t>Garlic ice cream flavor</t>
   </si>
   <si>
-    <t>icf:b868d0d7-e574-48b0-a6b2-433a01c7434a</t>
+    <t>icf:66</t>
   </si>
   <si>
     <t>Oyster</t>
@@ -2275,7 +2275,7 @@
     <t>Oyster ice cream flavor</t>
   </si>
   <si>
-    <t>icf:b023c80a-7d05-4324-8207-4e5bba5dec17</t>
+    <t>icf:67</t>
   </si>
   <si>
     <t>Korean Sweet corn</t>
@@ -2284,7 +2284,7 @@
     <t>Korean Sweet corn ice cream flavor</t>
   </si>
   <si>
-    <t>icf:96e04174-022b-4934-a431-3bb3f96f015f</t>
+    <t>icf:68</t>
   </si>
   <si>
     <t>Taro</t>
@@ -2293,7 +2293,7 @@
     <t>Taro ice cream flavor</t>
   </si>
   <si>
-    <t>icf:392def8f-2e32-4c23-ae4f-2f149787f3a6</t>
+    <t>icf:69</t>
   </si>
   <si>
     <t xml:space="preserve">Spundekas </t>
@@ -2302,7 +2302,7 @@
     <t>Ice cream flavor based on the German cream cheese of the same name</t>
   </si>
   <si>
-    <t>icf:8e63e629-3b8f-47d7-86d8-079bc74dc92c</t>
+    <t>icf:70</t>
   </si>
   <si>
     <t>Ube</t>
@@ -2323,7 +2323,7 @@
     <t>Savory ice cream flavors collection</t>
   </si>
   <si>
-    <t>http://vocab.example.com/icecreamflavors/collection/fruit</t>
+    <t>icf:1</t>
   </si>
   <si>
     <t>Taken from Wikipedia</t>
@@ -2332,7 +2332,10 @@
     <t>http://vocab.example.com/icecreamflavors/collection/choc-etc</t>
   </si>
   <si>
-    <t>http://vocab.example.com/icecreamflavors/collection/savory</t>
+    <t>icf:58</t>
+  </si>
+  <si>
+    <t>icf:22</t>
   </si>
 </sst>
 </file>
@@ -7891,9 +7894,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65B2936F-06B6-364A-893D-D48542B6FA7F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns6="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{65B2936F-06B6-364A-893D-D48542B6FA7F}">
   <dimension ref="A1:L71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18" ns3:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="49.1640625" style="21" customWidth="1"/>
     <col min="2" max="2" width="58.33203125" style="21" customWidth="1"/>
@@ -7908,7 +7911,7 @@
     <col min="13" max="16384" width="10.83203125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" ht="40" customHeight="1" ns3:dyDescent="0.15">
       <c r="A1" s="67" t="s">
         <v>13</v>
       </c>
@@ -7920,7 +7923,7 @@
       <c r="G1" s="67"/>
       <c r="H1" s="67"/>
     </row>
-    <row r="2" spans="1:12" ht="19" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:12" ht="19" ns3:dyDescent="0.15">
       <c r="A2" s="32" t="s">
         <v>56</v>
       </c>
@@ -7958,7 +7961,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="271" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:12" ht="271" customHeight="1" ns3:dyDescent="0.15">
       <c r="A3" s="27" t="s">
         <v>183</v>
       </c>
@@ -7996,7 +7999,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ns3:dyDescent="0.2">
       <c r="A4" s="59" t="s">
         <v>199</v>
       </c>
@@ -8009,7 +8012,7 @@
       <c r="D4" s="59"/>
       <c r="G4" s="20"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ns3:dyDescent="0.2">
       <c r="A5" s="59" t="s">
         <v>202</v>
       </c>
@@ -8023,7 +8026,7 @@
       <c r="G5" s="20"/>
       <c r="K5" s="20"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ns3:dyDescent="0.2">
       <c r="A6" s="59" t="s">
         <v>205</v>
       </c>
@@ -8038,7 +8041,7 @@
       </c>
       <c r="G6" s="56"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ns3:dyDescent="0.2">
       <c r="A7" s="59" t="s">
         <v>209</v>
       </c>
@@ -8051,7 +8054,7 @@
       <c r="D7" s="59"/>
       <c r="G7" s="56"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ns3:dyDescent="0.2">
       <c r="A8" s="59" t="s">
         <v>212</v>
       </c>
@@ -8064,7 +8067,7 @@
       <c r="D8" s="59"/>
       <c r="G8" s="20"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ns3:dyDescent="0.2">
       <c r="A9" s="59" t="s">
         <v>215</v>
       </c>
@@ -8077,7 +8080,7 @@
       <c r="D9" s="59"/>
       <c r="G9" s="56"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ns3:dyDescent="0.2">
       <c r="A10" s="59" t="s">
         <v>218</v>
       </c>
@@ -8090,7 +8093,7 @@
       <c r="D10" s="59"/>
       <c r="G10" s="56"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ns3:dyDescent="0.2">
       <c r="A11" s="59" t="s">
         <v>220</v>
       </c>
@@ -8103,7 +8106,7 @@
       <c r="D11" s="59"/>
       <c r="G11" s="56"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ns3:dyDescent="0.2">
       <c r="A12" s="59" t="s">
         <v>223</v>
       </c>
@@ -8116,7 +8119,7 @@
       <c r="D12" s="59"/>
       <c r="G12" s="20"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ns3:dyDescent="0.2">
       <c r="A13" s="59" t="s">
         <v>226</v>
       </c>
@@ -8129,7 +8132,7 @@
       <c r="D13" s="59"/>
       <c r="G13" s="20"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ns3:dyDescent="0.2">
       <c r="A14" s="59" t="s">
         <v>229</v>
       </c>
@@ -8142,7 +8145,7 @@
       <c r="D14" s="59"/>
       <c r="G14" s="56"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ns3:dyDescent="0.2">
       <c r="A15" s="59" t="s">
         <v>232</v>
       </c>
@@ -8155,7 +8158,7 @@
       <c r="D15" s="59"/>
       <c r="G15" s="56"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ns3:dyDescent="0.2">
       <c r="A16" s="59" t="s">
         <v>235</v>
       </c>
@@ -8169,7 +8172,7 @@
       <c r="E16" s="44"/>
       <c r="G16" s="20"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ns3:dyDescent="0.2">
       <c r="A17" s="59" t="s">
         <v>238</v>
       </c>
@@ -8183,7 +8186,7 @@
       <c r="E17" s="44"/>
       <c r="G17" s="56"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ns3:dyDescent="0.2">
       <c r="A18" s="59" t="s">
         <v>241</v>
       </c>
@@ -8196,7 +8199,7 @@
       <c r="D18" s="59"/>
       <c r="G18" s="20"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ns3:dyDescent="0.2">
       <c r="A19" s="59" t="s">
         <v>244</v>
       </c>
@@ -8209,7 +8212,7 @@
       <c r="D19" s="59"/>
       <c r="G19" s="20"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ns3:dyDescent="0.2">
       <c r="A20" s="59" t="s">
         <v>247</v>
       </c>
@@ -8222,7 +8225,7 @@
       <c r="D20" s="59"/>
       <c r="G20" s="20"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ns3:dyDescent="0.2">
       <c r="A21" s="59" t="s">
         <v>250</v>
       </c>
@@ -8235,7 +8238,7 @@
       <c r="D21" s="59"/>
       <c r="G21" s="20"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ns3:dyDescent="0.2">
       <c r="A22" s="59" t="s">
         <v>253</v>
       </c>
@@ -8248,7 +8251,7 @@
       <c r="D22" s="59"/>
       <c r="G22" s="20"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ns3:dyDescent="0.2">
       <c r="A23" s="59" t="s">
         <v>256</v>
       </c>
@@ -8261,7 +8264,7 @@
       <c r="D23" s="59"/>
       <c r="G23" s="20"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ns3:dyDescent="0.2">
       <c r="A24" s="59" t="s">
         <v>259</v>
       </c>
@@ -8274,7 +8277,7 @@
       <c r="D24" s="59"/>
       <c r="G24" s="20"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ns3:dyDescent="0.2">
       <c r="A25" s="59" t="s">
         <v>262</v>
       </c>
@@ -8287,7 +8290,7 @@
       <c r="D25" s="59"/>
       <c r="G25" s="20"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ns3:dyDescent="0.2">
       <c r="A26" s="59" t="s">
         <v>265</v>
       </c>
@@ -8300,7 +8303,7 @@
       <c r="D26" s="59"/>
       <c r="G26" s="20"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ns3:dyDescent="0.2">
       <c r="A27" s="59" t="s">
         <v>268</v>
       </c>
@@ -8313,7 +8316,7 @@
       <c r="D27" s="59"/>
       <c r="G27" s="20"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ns3:dyDescent="0.2">
       <c r="A28" s="59" t="s">
         <v>271</v>
       </c>
@@ -8326,7 +8329,7 @@
       <c r="D28" s="59"/>
       <c r="G28" s="20"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ns3:dyDescent="0.2">
       <c r="A29" s="59" t="s">
         <v>274</v>
       </c>
@@ -8339,7 +8342,7 @@
       <c r="D29" s="59"/>
       <c r="G29" s="20"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" ns3:dyDescent="0.2">
       <c r="A30" s="59" t="s">
         <v>277</v>
       </c>
@@ -8352,7 +8355,7 @@
       <c r="D30" s="59"/>
       <c r="G30" s="20"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" ns3:dyDescent="0.2">
       <c r="A31" s="59" t="s">
         <v>280</v>
       </c>
@@ -8365,7 +8368,7 @@
       <c r="D31" s="59"/>
       <c r="G31" s="20"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" ns3:dyDescent="0.2">
       <c r="A32" s="59" t="s">
         <v>283</v>
       </c>
@@ -8378,7 +8381,7 @@
       <c r="D32" s="59"/>
       <c r="G32" s="20"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" ns3:dyDescent="0.2">
       <c r="A33" s="59" t="s">
         <v>286</v>
       </c>
@@ -8391,7 +8394,7 @@
       <c r="D33" s="59"/>
       <c r="G33" s="20"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" ns3:dyDescent="0.2">
       <c r="A34" s="59" t="s">
         <v>289</v>
       </c>
@@ -8404,7 +8407,7 @@
       <c r="D34" s="59"/>
       <c r="G34" s="20"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ns3:dyDescent="0.2">
       <c r="A35" s="59" t="s">
         <v>292</v>
       </c>
@@ -8417,7 +8420,7 @@
       <c r="D35" s="59"/>
       <c r="G35" s="20"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" ns3:dyDescent="0.2">
       <c r="A36" s="59" t="s">
         <v>295</v>
       </c>
@@ -8430,7 +8433,7 @@
       <c r="D36" s="59"/>
       <c r="G36" s="20"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" ns3:dyDescent="0.2">
       <c r="A37" s="59" t="s">
         <v>298</v>
       </c>
@@ -8443,7 +8446,7 @@
       <c r="D37" s="59"/>
       <c r="G37" s="20"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" ns3:dyDescent="0.2">
       <c r="A38" s="59" t="s">
         <v>301</v>
       </c>
@@ -8456,7 +8459,7 @@
       <c r="D38" s="59"/>
       <c r="G38" s="20"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ns3:dyDescent="0.2">
       <c r="A39" s="59" t="s">
         <v>304</v>
       </c>
@@ -8469,7 +8472,7 @@
       <c r="D39" s="59"/>
       <c r="G39" s="20"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" ns3:dyDescent="0.2">
       <c r="A40" s="59" t="s">
         <v>307</v>
       </c>
@@ -8482,7 +8485,7 @@
       <c r="D40" s="59"/>
       <c r="G40" s="20"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" ns3:dyDescent="0.2">
       <c r="A41" s="59" t="s">
         <v>310</v>
       </c>
@@ -8495,7 +8498,7 @@
       <c r="D41" s="59"/>
       <c r="G41" s="20"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" ns3:dyDescent="0.2">
       <c r="A42" s="59" t="s">
         <v>313</v>
       </c>
@@ -8508,7 +8511,7 @@
       <c r="D42" s="59"/>
       <c r="G42" s="20"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" ns3:dyDescent="0.2">
       <c r="A43" s="59" t="s">
         <v>316</v>
       </c>
@@ -8521,7 +8524,7 @@
       <c r="D43" s="59"/>
       <c r="G43" s="20"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" ns3:dyDescent="0.2">
       <c r="A44" s="59" t="s">
         <v>319</v>
       </c>
@@ -8534,7 +8537,7 @@
       <c r="D44" s="59"/>
       <c r="G44" s="20"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" ns3:dyDescent="0.2">
       <c r="A45" s="59" t="s">
         <v>322</v>
       </c>
@@ -8547,7 +8550,7 @@
       <c r="D45" s="59"/>
       <c r="G45" s="20"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" ns3:dyDescent="0.2">
       <c r="A46" s="59" t="s">
         <v>325</v>
       </c>
@@ -8560,7 +8563,7 @@
       <c r="D46" s="59"/>
       <c r="G46" s="20"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" ns3:dyDescent="0.2">
       <c r="A47" s="59" t="s">
         <v>328</v>
       </c>
@@ -8573,7 +8576,7 @@
       <c r="D47" s="59"/>
       <c r="G47" s="20"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" ns3:dyDescent="0.2">
       <c r="A48" s="59" t="s">
         <v>331</v>
       </c>
@@ -8586,7 +8589,7 @@
       <c r="D48" s="59"/>
       <c r="G48" s="20"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" ns3:dyDescent="0.2">
       <c r="A49" s="59" t="s">
         <v>334</v>
       </c>
@@ -8599,7 +8602,7 @@
       <c r="D49" s="59"/>
       <c r="G49" s="20"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ns3:dyDescent="0.2">
       <c r="A50" s="59" t="s">
         <v>337</v>
       </c>
@@ -8612,7 +8615,7 @@
       <c r="D50" s="59"/>
       <c r="G50" s="20"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" ns3:dyDescent="0.2">
       <c r="A51" s="59" t="s">
         <v>340</v>
       </c>
@@ -8625,7 +8628,7 @@
       <c r="D51" s="59"/>
       <c r="G51" s="20"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" ns3:dyDescent="0.2">
       <c r="A52" s="59" t="s">
         <v>343</v>
       </c>
@@ -8637,7 +8640,7 @@
       </c>
       <c r="D52" s="59"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" ns3:dyDescent="0.2">
       <c r="A53" s="59" t="s">
         <v>346</v>
       </c>
@@ -8649,7 +8652,7 @@
       </c>
       <c r="D53" s="59"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" ns3:dyDescent="0.2">
       <c r="A54" s="59" t="s">
         <v>349</v>
       </c>
@@ -8661,7 +8664,7 @@
       </c>
       <c r="D54" s="59"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" ns3:dyDescent="0.2">
       <c r="A55" s="59" t="s">
         <v>352</v>
       </c>
@@ -8673,7 +8676,7 @@
       </c>
       <c r="D55" s="59"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" ns3:dyDescent="0.2">
       <c r="A56" s="59" t="s">
         <v>355</v>
       </c>
@@ -8685,7 +8688,7 @@
       </c>
       <c r="D56" s="59"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" ns3:dyDescent="0.2">
       <c r="A57" s="59" t="s">
         <v>358</v>
       </c>
@@ -8697,7 +8700,7 @@
       </c>
       <c r="D57" s="59"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" ns3:dyDescent="0.2">
       <c r="A58" s="59" t="s">
         <v>361</v>
       </c>
@@ -8709,7 +8712,7 @@
       </c>
       <c r="D58" s="59"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ns3:dyDescent="0.2">
       <c r="A59" s="59" t="s">
         <v>365</v>
       </c>
@@ -8721,7 +8724,7 @@
       </c>
       <c r="D59" s="59"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" ns3:dyDescent="0.2">
       <c r="A60" s="59" t="s">
         <v>368</v>
       </c>
@@ -8733,7 +8736,7 @@
       </c>
       <c r="D60" s="59"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" ns3:dyDescent="0.2">
       <c r="A61" s="59" t="s">
         <v>371</v>
       </c>
@@ -8745,7 +8748,7 @@
       </c>
       <c r="D61" s="59"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ns3:dyDescent="0.2">
       <c r="A62" s="59" t="s">
         <v>374</v>
       </c>
@@ -8757,7 +8760,7 @@
       </c>
       <c r="D62" s="59"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" ns3:dyDescent="0.2">
       <c r="A63" s="59" t="s">
         <v>377</v>
       </c>
@@ -8769,7 +8772,7 @@
       </c>
       <c r="D63" s="59"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" ns3:dyDescent="0.2">
       <c r="A64" s="59" t="s">
         <v>380</v>
       </c>
@@ -8781,7 +8784,7 @@
       </c>
       <c r="D64" s="59"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" ns3:dyDescent="0.2">
       <c r="A65" s="59" t="s">
         <v>383</v>
       </c>
@@ -8793,7 +8796,7 @@
       </c>
       <c r="D65" s="59"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" ns3:dyDescent="0.2">
       <c r="A66" s="59" t="s">
         <v>386</v>
       </c>
@@ -8805,7 +8808,7 @@
       </c>
       <c r="D66" s="59"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" ns3:dyDescent="0.2">
       <c r="A67" s="59" t="s">
         <v>389</v>
       </c>
@@ -8817,7 +8820,7 @@
       </c>
       <c r="D67" s="59"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" ns3:dyDescent="0.2">
       <c r="A68" s="59" t="s">
         <v>392</v>
       </c>
@@ -8829,7 +8832,7 @@
       </c>
       <c r="D68" s="59"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" ns3:dyDescent="0.2">
       <c r="A69" s="59" t="s">
         <v>395</v>
       </c>
@@ -8841,7 +8844,7 @@
       </c>
       <c r="D69" s="59"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" ns3:dyDescent="0.2">
       <c r="A70" s="59" t="s">
         <v>398</v>
       </c>
@@ -8855,7 +8858,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:4" ns3:dyDescent="0.15">
       <c r="A71" s="61"/>
       <c r="B71" s="61"/>
       <c r="C71" s="62"/>
@@ -8869,15 +8872,15 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ACD342F2-949F-8E4F-8019-9523BB9FDCE8}">
-          <x14:formula1>
-            <xm:f>Lookups!$A$3:$A$16</xm:f>
-          </x14:formula1>
-          <xm:sqref>I4:I29</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns5:dataValidations count="1">
+        <ns5:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" ns2:uid="{ACD342F2-949F-8E4F-8019-9523BB9FDCE8}">
+          <ns5:formula1>
+            <ns6:f>Lookups!$A$3:$A$16</ns6:f>
+          </ns5:formula1>
+          <ns6:sqref>I4:I29</ns6:sqref>
+        </ns5:dataValidation>
+      </ns5:dataValidations>
     </ext>
   </extLst>
 </worksheet>
@@ -9023,12 +9026,12 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G193"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="20" customHeight="1" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="83.1640625" style="19" customWidth="1"/>
     <col min="2" max="2" width="23.6640625" style="19" customWidth="1"/>
@@ -9040,7 +9043,7 @@
     <col min="8" max="16384" width="12.5" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="40" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="64" t="s">
         <v>18</v>
       </c>
@@ -9049,7 +9052,7 @@
       <c r="D1" s="65"/>
       <c r="E1" s="65"/>
     </row>
-    <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A2" s="28" t="s">
         <v>57</v>
       </c>
@@ -9066,7 +9069,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="114" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="114" ns3:dyDescent="0.2">
       <c r="A3" s="54"/>
       <c r="B3" s="55" t="s">
         <v>146</v>
@@ -9081,7 +9084,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="21" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="21" customFormat="1" ht="19" ns3:dyDescent="0.25">
       <c r="A4" s="63" t="s">
         <v>405</v>
       </c>
@@ -9098,7 +9101,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="19" ns3:dyDescent="0.25">
       <c r="A5" s="63" t="s">
         <v>405</v>
       </c>
@@ -9113,7 +9116,7 @@
       </c>
       <c r="E5" s="18"/>
     </row>
-    <row r="6" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A6" s="63" t="s">
         <v>405</v>
       </c>
@@ -9128,7 +9131,7 @@
       </c>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A7" s="63" t="s">
         <v>405</v>
       </c>
@@ -9143,7 +9146,7 @@
       </c>
       <c r="E7" s="18"/>
     </row>
-    <row r="8" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A8" s="63" t="s">
         <v>405</v>
       </c>
@@ -9160,7 +9163,7 @@
       <c r="F8" s="42"/>
       <c r="G8" s="42"/>
     </row>
-    <row r="9" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A9" s="63" t="s">
         <v>405</v>
       </c>
@@ -9177,7 +9180,7 @@
       <c r="F9" s="37"/>
       <c r="G9" s="43"/>
     </row>
-    <row r="10" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A10" s="63" t="s">
         <v>405</v>
       </c>
@@ -9194,7 +9197,7 @@
       <c r="F10" s="37"/>
       <c r="G10" s="43"/>
     </row>
-    <row r="11" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A11" s="63" t="s">
         <v>405</v>
       </c>
@@ -9211,7 +9214,7 @@
       <c r="F11" s="37"/>
       <c r="G11" s="43"/>
     </row>
-    <row r="12" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A12" s="63" t="s">
         <v>405</v>
       </c>
@@ -9228,7 +9231,7 @@
       <c r="F12" s="37"/>
       <c r="G12" s="43"/>
     </row>
-    <row r="13" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A13" s="63" t="s">
         <v>405</v>
       </c>
@@ -9245,7 +9248,7 @@
       <c r="F13" s="37"/>
       <c r="G13" s="43"/>
     </row>
-    <row r="14" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A14" s="63" t="s">
         <v>405</v>
       </c>
@@ -9262,7 +9265,7 @@
       <c r="F14" s="37"/>
       <c r="G14" s="43"/>
     </row>
-    <row r="15" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A15" s="63" t="s">
         <v>405</v>
       </c>
@@ -9279,7 +9282,7 @@
       <c r="F15" s="37"/>
       <c r="G15" s="43"/>
     </row>
-    <row r="16" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A16" s="63" t="s">
         <v>405</v>
       </c>
@@ -9296,7 +9299,7 @@
       <c r="F16" s="37"/>
       <c r="G16" s="43"/>
     </row>
-    <row r="17" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A17" s="63" t="s">
         <v>405</v>
       </c>
@@ -9313,7 +9316,7 @@
       <c r="F17" s="37"/>
       <c r="G17" s="43"/>
     </row>
-    <row r="18" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A18" s="63" t="s">
         <v>405</v>
       </c>
@@ -9330,7 +9333,7 @@
       <c r="F18" s="19"/>
       <c r="G18" s="19"/>
     </row>
-    <row r="19" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A19" s="63" t="s">
         <v>405</v>
       </c>
@@ -9347,7 +9350,7 @@
       <c r="F19" s="19"/>
       <c r="G19" s="19"/>
     </row>
-    <row r="20" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A20" s="63" t="s">
         <v>405</v>
       </c>
@@ -9364,7 +9367,7 @@
       <c r="F20" s="19"/>
       <c r="G20" s="19"/>
     </row>
-    <row r="21" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A21" s="63" t="s">
         <v>405</v>
       </c>
@@ -9381,7 +9384,7 @@
       <c r="F21" s="19"/>
       <c r="G21" s="19"/>
     </row>
-    <row r="22" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A22" s="63" t="s">
         <v>405</v>
       </c>
@@ -9398,7 +9401,7 @@
       <c r="F22" s="19"/>
       <c r="G22" s="19"/>
     </row>
-    <row r="23" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A23" s="63" t="s">
         <v>405</v>
       </c>
@@ -9415,9 +9418,9 @@
       <c r="F23" s="19"/>
       <c r="G23" s="19"/>
     </row>
-    <row r="24" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A24" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B24" s="63" t="s">
         <v>258</v>
@@ -9434,9 +9437,9 @@
       <c r="F24" s="19"/>
       <c r="G24" s="19"/>
     </row>
-    <row r="25" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A25" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B25" s="63" t="s">
         <v>258</v>
@@ -9451,9 +9454,9 @@
       <c r="F25" s="19"/>
       <c r="G25" s="19"/>
     </row>
-    <row r="26" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A26" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B26" s="63" t="s">
         <v>258</v>
@@ -9468,9 +9471,9 @@
       <c r="F26" s="19"/>
       <c r="G26" s="19"/>
     </row>
-    <row r="27" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A27" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B27" s="63" t="s">
         <v>258</v>
@@ -9485,9 +9488,9 @@
       <c r="F27" s="19"/>
       <c r="G27" s="19"/>
     </row>
-    <row r="28" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A28" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B28" s="63" t="s">
         <v>258</v>
@@ -9502,9 +9505,9 @@
       <c r="F28" s="19"/>
       <c r="G28" s="19"/>
     </row>
-    <row r="29" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A29" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B29" s="63" t="s">
         <v>258</v>
@@ -9519,9 +9522,9 @@
       <c r="F29" s="19"/>
       <c r="G29" s="19"/>
     </row>
-    <row r="30" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A30" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B30" s="63" t="s">
         <v>258</v>
@@ -9536,9 +9539,9 @@
       <c r="F30" s="19"/>
       <c r="G30" s="19"/>
     </row>
-    <row r="31" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A31" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B31" s="63" t="s">
         <v>258</v>
@@ -9553,9 +9556,9 @@
       <c r="F31" s="19"/>
       <c r="G31" s="19"/>
     </row>
-    <row r="32" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A32" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B32" s="63" t="s">
         <v>258</v>
@@ -9570,9 +9573,9 @@
       <c r="F32" s="19"/>
       <c r="G32" s="19"/>
     </row>
-    <row r="33" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A33" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B33" s="63" t="s">
         <v>258</v>
@@ -9587,9 +9590,9 @@
       <c r="F33" s="19"/>
       <c r="G33" s="19"/>
     </row>
-    <row r="34" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A34" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B34" s="63" t="s">
         <v>258</v>
@@ -9604,9 +9607,9 @@
       <c r="F34" s="19"/>
       <c r="G34" s="19"/>
     </row>
-    <row r="35" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A35" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B35" s="63" t="s">
         <v>258</v>
@@ -9621,9 +9624,9 @@
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
     </row>
-    <row r="36" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A36" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B36" s="63" t="s">
         <v>258</v>
@@ -9636,9 +9639,9 @@
       </c>
       <c r="E36" s="18"/>
     </row>
-    <row r="37" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A37" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B37" s="63" t="s">
         <v>258</v>
@@ -9651,9 +9654,9 @@
       </c>
       <c r="E37" s="18"/>
     </row>
-    <row r="38" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A38" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B38" s="63" t="s">
         <v>258</v>
@@ -9666,9 +9669,9 @@
       </c>
       <c r="E38" s="18"/>
     </row>
-    <row r="39" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A39" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B39" s="63" t="s">
         <v>258</v>
@@ -9681,9 +9684,9 @@
       </c>
       <c r="E39" s="18"/>
     </row>
-    <row r="40" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A40" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B40" s="63" t="s">
         <v>258</v>
@@ -9696,9 +9699,9 @@
       </c>
       <c r="E40" s="18"/>
     </row>
-    <row r="41" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A41" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B41" s="63" t="s">
         <v>258</v>
@@ -9711,9 +9714,9 @@
       </c>
       <c r="E41" s="18"/>
     </row>
-    <row r="42" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A42" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B42" s="63" t="s">
         <v>258</v>
@@ -9726,9 +9729,9 @@
       </c>
       <c r="E42" s="18"/>
     </row>
-    <row r="43" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A43" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B43" s="63" t="s">
         <v>258</v>
@@ -9741,9 +9744,9 @@
       </c>
       <c r="E43" s="18"/>
     </row>
-    <row r="44" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A44" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B44" s="63" t="s">
         <v>258</v>
@@ -9756,9 +9759,9 @@
       </c>
       <c r="E44" s="18"/>
     </row>
-    <row r="45" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A45" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B45" s="63" t="s">
         <v>258</v>
@@ -9771,9 +9774,9 @@
       </c>
       <c r="E45"/>
     </row>
-    <row r="46" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A46" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B46" s="63" t="s">
         <v>258</v>
@@ -9786,9 +9789,9 @@
       </c>
       <c r="E46" s="18"/>
     </row>
-    <row r="47" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A47" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B47" s="63" t="s">
         <v>258</v>
@@ -9801,9 +9804,9 @@
       </c>
       <c r="E47" s="18"/>
     </row>
-    <row r="48" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A48" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B48" s="63" t="s">
         <v>258</v>
@@ -9816,9 +9819,9 @@
       </c>
       <c r="E48" s="18"/>
     </row>
-    <row r="49" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A49" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B49" s="63" t="s">
         <v>258</v>
@@ -9831,9 +9834,9 @@
       </c>
       <c r="E49" s="18"/>
     </row>
-    <row r="50" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A50" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B50" s="63" t="s">
         <v>258</v>
@@ -9846,9 +9849,9 @@
       </c>
       <c r="E50" s="18"/>
     </row>
-    <row r="51" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A51" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B51" s="63" t="s">
         <v>258</v>
@@ -9861,9 +9864,9 @@
       </c>
       <c r="E51" s="18"/>
     </row>
-    <row r="52" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A52" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B52" s="63" t="s">
         <v>258</v>
@@ -9876,9 +9879,9 @@
       </c>
       <c r="E52" s="18"/>
     </row>
-    <row r="53" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A53" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B53" s="63" t="s">
         <v>258</v>
@@ -9891,9 +9894,9 @@
       </c>
       <c r="E53" s="18"/>
     </row>
-    <row r="54" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A54" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B54" s="63" t="s">
         <v>258</v>
@@ -9906,9 +9909,9 @@
       </c>
       <c r="E54"/>
     </row>
-    <row r="55" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A55" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B55" s="63" t="s">
         <v>258</v>
@@ -9921,9 +9924,9 @@
       </c>
       <c r="E55" s="18"/>
     </row>
-    <row r="56" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A56" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B56" s="63" t="s">
         <v>258</v>
@@ -9936,9 +9939,9 @@
       </c>
       <c r="E56" s="18"/>
     </row>
-    <row r="57" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A57" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B57" s="63" t="s">
         <v>258</v>
@@ -9951,9 +9954,9 @@
       </c>
       <c r="E57" s="18"/>
     </row>
-    <row r="58" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A58" s="63" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B58" s="63" t="s">
         <v>258</v>
@@ -9966,7 +9969,7 @@
       </c>
       <c r="E58" s="18"/>
     </row>
-    <row r="59" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A59" s="63" t="s">
         <v>408</v>
       </c>
@@ -9983,7 +9986,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A60" s="63" t="s">
         <v>408</v>
       </c>
@@ -9998,7 +10001,7 @@
       </c>
       <c r="E60" s="18"/>
     </row>
-    <row r="61" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A61" s="63" t="s">
         <v>408</v>
       </c>
@@ -10013,7 +10016,7 @@
       </c>
       <c r="E61" s="18"/>
     </row>
-    <row r="62" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A62" s="63" t="s">
         <v>408</v>
       </c>
@@ -10028,7 +10031,7 @@
       </c>
       <c r="E62"/>
     </row>
-    <row r="63" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A63" s="63" t="s">
         <v>408</v>
       </c>
@@ -10043,7 +10046,7 @@
       </c>
       <c r="E63" s="18"/>
     </row>
-    <row r="64" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A64" s="63" t="s">
         <v>408</v>
       </c>
@@ -10058,7 +10061,7 @@
       </c>
       <c r="E64" s="18"/>
     </row>
-    <row r="65" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A65" s="63" t="s">
         <v>408</v>
       </c>
@@ -10073,7 +10076,7 @@
       </c>
       <c r="E65" s="18"/>
     </row>
-    <row r="66" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A66" s="63" t="s">
         <v>408</v>
       </c>
@@ -10088,7 +10091,7 @@
       </c>
       <c r="E66"/>
     </row>
-    <row r="67" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A67" s="63" t="s">
         <v>408</v>
       </c>
@@ -10103,7 +10106,7 @@
       </c>
       <c r="E67"/>
     </row>
-    <row r="68" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A68" s="63" t="s">
         <v>408</v>
       </c>
@@ -10118,7 +10121,7 @@
       </c>
       <c r="E68" s="18"/>
     </row>
-    <row r="69" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A69" s="63" t="s">
         <v>408</v>
       </c>
@@ -10133,7 +10136,7 @@
       </c>
       <c r="E69" s="18"/>
     </row>
-    <row r="70" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A70" s="63" t="s">
         <v>408</v>
       </c>
@@ -10148,861 +10151,861 @@
       </c>
       <c r="E70" s="18"/>
     </row>
-    <row r="71" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A71" s="31"/>
       <c r="B71" s="31"/>
       <c r="C71" s="31"/>
       <c r="D71" s="63"/>
       <c r="E71" s="31"/>
     </row>
-    <row r="72" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A72" s="31"/>
       <c r="B72" s="31"/>
       <c r="C72" s="31"/>
       <c r="D72" s="63"/>
       <c r="E72" s="31"/>
     </row>
-    <row r="73" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A73" s="31"/>
       <c r="B73" s="31"/>
       <c r="C73" s="31"/>
       <c r="D73" s="63"/>
       <c r="E73" s="31"/>
     </row>
-    <row r="74" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.25">
       <c r="A74" s="31"/>
       <c r="B74" s="31"/>
       <c r="C74" s="31"/>
       <c r="D74" s="63"/>
       <c r="E74" s="31"/>
     </row>
-    <row r="75" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A75" s="31"/>
       <c r="B75" s="31"/>
       <c r="C75" s="31"/>
       <c r="D75" s="31"/>
       <c r="E75" s="31"/>
     </row>
-    <row r="76" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A76" s="31"/>
       <c r="B76" s="31"/>
       <c r="C76" s="31"/>
       <c r="D76" s="31"/>
       <c r="E76" s="31"/>
     </row>
-    <row r="77" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A77" s="31"/>
       <c r="B77" s="31"/>
       <c r="C77" s="31"/>
       <c r="D77" s="31"/>
       <c r="E77" s="31"/>
     </row>
-    <row r="78" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A78" s="31"/>
       <c r="B78" s="31"/>
       <c r="C78" s="31"/>
       <c r="D78" s="31"/>
       <c r="E78" s="31"/>
     </row>
-    <row r="79" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A79" s="31"/>
       <c r="B79" s="31"/>
       <c r="C79" s="31"/>
       <c r="D79" s="31"/>
       <c r="E79" s="31"/>
     </row>
-    <row r="80" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A80" s="31"/>
       <c r="B80" s="31"/>
       <c r="C80" s="31"/>
       <c r="D80" s="31"/>
       <c r="E80" s="31"/>
     </row>
-    <row r="81" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A81" s="31"/>
       <c r="B81" s="31"/>
       <c r="C81" s="31"/>
       <c r="D81" s="31"/>
       <c r="E81" s="31"/>
     </row>
-    <row r="82" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A82" s="31"/>
       <c r="B82" s="31"/>
       <c r="C82" s="31"/>
       <c r="D82" s="31"/>
       <c r="E82" s="31"/>
     </row>
-    <row r="83" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A83" s="31"/>
       <c r="B83" s="31"/>
       <c r="C83" s="31"/>
       <c r="D83" s="31"/>
       <c r="E83" s="31"/>
     </row>
-    <row r="84" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A84" s="31"/>
       <c r="B84" s="31"/>
       <c r="C84" s="31"/>
       <c r="D84" s="31"/>
       <c r="E84" s="31"/>
     </row>
-    <row r="85" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A85" s="31"/>
       <c r="B85" s="31"/>
       <c r="C85" s="31"/>
       <c r="D85" s="31"/>
       <c r="E85" s="31"/>
     </row>
-    <row r="86" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A86" s="31"/>
       <c r="B86" s="31"/>
       <c r="C86" s="31"/>
       <c r="D86" s="31"/>
       <c r="E86" s="31"/>
     </row>
-    <row r="87" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A87" s="31"/>
       <c r="B87" s="31"/>
       <c r="C87" s="31"/>
       <c r="D87" s="31"/>
       <c r="E87" s="31"/>
     </row>
-    <row r="88" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A88" s="31"/>
       <c r="B88" s="31"/>
       <c r="C88" s="31"/>
       <c r="D88" s="31"/>
       <c r="E88" s="31"/>
     </row>
-    <row r="89" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A89" s="31"/>
       <c r="B89" s="31"/>
       <c r="C89" s="31"/>
       <c r="D89" s="31"/>
       <c r="E89" s="31"/>
     </row>
-    <row r="90" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A90" s="31"/>
       <c r="B90" s="31"/>
       <c r="C90" s="31"/>
       <c r="D90" s="31"/>
       <c r="E90" s="31"/>
     </row>
-    <row r="91" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A91" s="31"/>
       <c r="B91" s="31"/>
       <c r="C91" s="31"/>
       <c r="D91" s="31"/>
       <c r="E91" s="31"/>
     </row>
-    <row r="92" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A92" s="31"/>
       <c r="B92" s="31"/>
       <c r="C92" s="31"/>
       <c r="D92" s="31"/>
       <c r="E92" s="31"/>
     </row>
-    <row r="93" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A93" s="31"/>
       <c r="B93" s="31"/>
       <c r="C93" s="31"/>
       <c r="D93" s="31"/>
       <c r="E93" s="31"/>
     </row>
-    <row r="94" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A94" s="31"/>
       <c r="B94" s="31"/>
       <c r="C94" s="31"/>
       <c r="D94" s="31"/>
       <c r="E94" s="31"/>
     </row>
-    <row r="95" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A95" s="31"/>
       <c r="B95" s="31"/>
       <c r="C95" s="31"/>
       <c r="D95" s="31"/>
       <c r="E95" s="31"/>
     </row>
-    <row r="96" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A96" s="31"/>
       <c r="B96" s="31"/>
       <c r="C96" s="31"/>
       <c r="D96" s="31"/>
       <c r="E96" s="31"/>
     </row>
-    <row r="97" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A97" s="31"/>
       <c r="B97" s="31"/>
       <c r="C97" s="31"/>
       <c r="D97" s="31"/>
       <c r="E97" s="31"/>
     </row>
-    <row r="98" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A98" s="31"/>
       <c r="B98" s="31"/>
       <c r="C98" s="31"/>
       <c r="D98" s="31"/>
       <c r="E98" s="31"/>
     </row>
-    <row r="99" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A99" s="31"/>
       <c r="B99" s="31"/>
       <c r="C99" s="31"/>
       <c r="D99" s="31"/>
       <c r="E99" s="31"/>
     </row>
-    <row r="100" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A100" s="31"/>
       <c r="B100" s="31"/>
       <c r="C100" s="31"/>
       <c r="D100" s="31"/>
       <c r="E100" s="31"/>
     </row>
-    <row r="101" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A101" s="31"/>
       <c r="B101" s="31"/>
       <c r="C101" s="31"/>
       <c r="D101" s="31"/>
       <c r="E101" s="31"/>
     </row>
-    <row r="102" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A102" s="31"/>
       <c r="B102" s="31"/>
       <c r="C102" s="31"/>
       <c r="D102" s="31"/>
       <c r="E102" s="31"/>
     </row>
-    <row r="103" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A103" s="31"/>
       <c r="B103" s="31"/>
       <c r="C103" s="31"/>
       <c r="D103" s="31"/>
       <c r="E103" s="31"/>
     </row>
-    <row r="104" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A104" s="31"/>
       <c r="B104" s="31"/>
       <c r="C104" s="31"/>
       <c r="D104" s="31"/>
       <c r="E104" s="31"/>
     </row>
-    <row r="105" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A105" s="31"/>
       <c r="B105" s="31"/>
       <c r="C105" s="31"/>
       <c r="D105" s="31"/>
       <c r="E105" s="31"/>
     </row>
-    <row r="106" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A106" s="31"/>
       <c r="B106" s="31"/>
       <c r="C106" s="31"/>
       <c r="D106" s="31"/>
       <c r="E106" s="31"/>
     </row>
-    <row r="107" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A107" s="31"/>
       <c r="B107" s="31"/>
       <c r="C107" s="31"/>
       <c r="D107" s="31"/>
       <c r="E107" s="31"/>
     </row>
-    <row r="108" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A108" s="31"/>
       <c r="B108" s="31"/>
       <c r="C108" s="31"/>
       <c r="D108" s="31"/>
       <c r="E108" s="31"/>
     </row>
-    <row r="109" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A109" s="31"/>
       <c r="B109" s="31"/>
       <c r="C109" s="31"/>
       <c r="D109" s="31"/>
       <c r="E109" s="31"/>
     </row>
-    <row r="110" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A110" s="31"/>
       <c r="B110" s="31"/>
       <c r="C110" s="31"/>
       <c r="D110" s="31"/>
       <c r="E110" s="31"/>
     </row>
-    <row r="111" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A111" s="31"/>
       <c r="B111" s="31"/>
       <c r="C111" s="31"/>
       <c r="D111" s="31"/>
       <c r="E111" s="31"/>
     </row>
-    <row r="112" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A112" s="31"/>
       <c r="B112" s="31"/>
       <c r="C112" s="31"/>
       <c r="D112" s="31"/>
       <c r="E112" s="31"/>
     </row>
-    <row r="113" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A113" s="31"/>
       <c r="B113" s="31"/>
       <c r="C113" s="31"/>
       <c r="D113" s="31"/>
       <c r="E113" s="31"/>
     </row>
-    <row r="114" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A114" s="31"/>
       <c r="B114" s="31"/>
       <c r="C114" s="31"/>
       <c r="D114" s="31"/>
       <c r="E114" s="31"/>
     </row>
-    <row r="115" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A115" s="31"/>
       <c r="B115" s="31"/>
       <c r="C115" s="31"/>
       <c r="D115" s="31"/>
       <c r="E115" s="31"/>
     </row>
-    <row r="116" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A116" s="31"/>
       <c r="B116" s="31"/>
       <c r="C116" s="31"/>
       <c r="D116" s="31"/>
       <c r="E116" s="31"/>
     </row>
-    <row r="117" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A117" s="31"/>
       <c r="B117" s="31"/>
       <c r="C117" s="31"/>
       <c r="D117" s="31"/>
       <c r="E117" s="31"/>
     </row>
-    <row r="118" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A118" s="31"/>
       <c r="B118" s="31"/>
       <c r="C118" s="31"/>
       <c r="D118" s="31"/>
       <c r="E118" s="31"/>
     </row>
-    <row r="119" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A119" s="31"/>
       <c r="B119" s="31"/>
       <c r="C119" s="31"/>
       <c r="D119" s="31"/>
       <c r="E119" s="31"/>
     </row>
-    <row r="120" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A120" s="31"/>
       <c r="B120" s="31"/>
       <c r="C120" s="31"/>
       <c r="D120" s="31"/>
       <c r="E120" s="31"/>
     </row>
-    <row r="121" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A121" s="31"/>
       <c r="B121" s="31"/>
       <c r="C121" s="31"/>
       <c r="D121" s="31"/>
       <c r="E121" s="31"/>
     </row>
-    <row r="122" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A122" s="31"/>
       <c r="B122" s="31"/>
       <c r="C122" s="31"/>
       <c r="D122" s="31"/>
       <c r="E122" s="31"/>
     </row>
-    <row r="123" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A123" s="31"/>
       <c r="B123" s="31"/>
       <c r="C123" s="31"/>
       <c r="D123" s="31"/>
       <c r="E123" s="31"/>
     </row>
-    <row r="124" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A124" s="31"/>
       <c r="B124" s="31"/>
       <c r="C124" s="31"/>
       <c r="D124" s="31"/>
       <c r="E124" s="31"/>
     </row>
-    <row r="125" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A125" s="31"/>
       <c r="B125" s="31"/>
       <c r="C125" s="31"/>
       <c r="D125" s="31"/>
       <c r="E125" s="31"/>
     </row>
-    <row r="126" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A126" s="31"/>
       <c r="B126" s="31"/>
       <c r="C126" s="31"/>
       <c r="D126" s="31"/>
       <c r="E126" s="31"/>
     </row>
-    <row r="127" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A127" s="31"/>
       <c r="B127" s="31"/>
       <c r="C127" s="31"/>
       <c r="D127" s="31"/>
       <c r="E127" s="31"/>
     </row>
-    <row r="128" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A128" s="31"/>
       <c r="B128" s="31"/>
       <c r="C128" s="31"/>
       <c r="D128" s="31"/>
       <c r="E128" s="31"/>
     </row>
-    <row r="129" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A129" s="31"/>
       <c r="B129" s="31"/>
       <c r="C129" s="31"/>
       <c r="D129" s="31"/>
       <c r="E129" s="31"/>
     </row>
-    <row r="130" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A130" s="31"/>
       <c r="B130" s="31"/>
       <c r="C130" s="31"/>
       <c r="D130" s="31"/>
       <c r="E130" s="31"/>
     </row>
-    <row r="131" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A131" s="31"/>
       <c r="B131" s="31"/>
       <c r="C131" s="31"/>
       <c r="D131" s="31"/>
       <c r="E131" s="31"/>
     </row>
-    <row r="132" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A132" s="31"/>
       <c r="B132" s="31"/>
       <c r="C132" s="31"/>
       <c r="D132" s="31"/>
       <c r="E132" s="31"/>
     </row>
-    <row r="133" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A133" s="31"/>
       <c r="B133" s="31"/>
       <c r="C133" s="31"/>
       <c r="D133" s="31"/>
       <c r="E133" s="31"/>
     </row>
-    <row r="134" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A134" s="31"/>
       <c r="B134" s="31"/>
       <c r="C134" s="31"/>
       <c r="D134" s="31"/>
       <c r="E134" s="31"/>
     </row>
-    <row r="135" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A135" s="31"/>
       <c r="B135" s="31"/>
       <c r="C135" s="31"/>
       <c r="D135" s="31"/>
       <c r="E135" s="31"/>
     </row>
-    <row r="136" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A136" s="31"/>
       <c r="B136" s="31"/>
       <c r="C136" s="31"/>
       <c r="D136" s="31"/>
       <c r="E136" s="31"/>
     </row>
-    <row r="137" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A137" s="31"/>
       <c r="B137" s="31"/>
       <c r="C137" s="31"/>
       <c r="D137" s="31"/>
       <c r="E137" s="31"/>
     </row>
-    <row r="138" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A138" s="31"/>
       <c r="B138" s="31"/>
       <c r="C138" s="31"/>
       <c r="D138" s="31"/>
       <c r="E138" s="31"/>
     </row>
-    <row r="139" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A139" s="31"/>
       <c r="B139" s="31"/>
       <c r="C139" s="31"/>
       <c r="D139" s="31"/>
       <c r="E139" s="31"/>
     </row>
-    <row r="140" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A140" s="31"/>
       <c r="B140" s="31"/>
       <c r="C140" s="31"/>
       <c r="D140" s="31"/>
       <c r="E140" s="31"/>
     </row>
-    <row r="141" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A141" s="31"/>
       <c r="B141" s="31"/>
       <c r="C141" s="31"/>
       <c r="D141" s="31"/>
       <c r="E141" s="31"/>
     </row>
-    <row r="142" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A142" s="31"/>
       <c r="B142" s="31"/>
       <c r="C142" s="31"/>
       <c r="D142" s="31"/>
       <c r="E142" s="31"/>
     </row>
-    <row r="143" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A143" s="31"/>
       <c r="B143" s="31"/>
       <c r="C143" s="31"/>
       <c r="D143" s="31"/>
       <c r="E143" s="31"/>
     </row>
-    <row r="144" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A144" s="31"/>
       <c r="B144" s="31"/>
       <c r="C144" s="31"/>
       <c r="D144" s="31"/>
       <c r="E144" s="31"/>
     </row>
-    <row r="145" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A145" s="31"/>
       <c r="B145" s="31"/>
       <c r="C145" s="31"/>
       <c r="D145" s="31"/>
       <c r="E145" s="31"/>
     </row>
-    <row r="146" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A146" s="31"/>
       <c r="B146" s="31"/>
       <c r="C146" s="31"/>
       <c r="D146" s="31"/>
       <c r="E146" s="31"/>
     </row>
-    <row r="147" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A147" s="31"/>
       <c r="B147" s="31"/>
       <c r="C147" s="31"/>
       <c r="D147" s="31"/>
       <c r="E147" s="31"/>
     </row>
-    <row r="148" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A148" s="31"/>
       <c r="B148" s="31"/>
       <c r="C148" s="31"/>
       <c r="D148" s="31"/>
       <c r="E148" s="31"/>
     </row>
-    <row r="149" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A149" s="31"/>
       <c r="B149" s="31"/>
       <c r="C149" s="31"/>
       <c r="D149" s="31"/>
       <c r="E149" s="31"/>
     </row>
-    <row r="150" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A150" s="31"/>
       <c r="B150" s="31"/>
       <c r="C150" s="31"/>
       <c r="D150" s="31"/>
       <c r="E150" s="31"/>
     </row>
-    <row r="151" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A151" s="31"/>
       <c r="B151" s="31"/>
       <c r="C151" s="31"/>
       <c r="D151" s="31"/>
       <c r="E151" s="31"/>
     </row>
-    <row r="152" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A152" s="31"/>
       <c r="B152" s="31"/>
       <c r="C152" s="31"/>
       <c r="D152" s="31"/>
       <c r="E152" s="31"/>
     </row>
-    <row r="153" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A153" s="31"/>
       <c r="B153" s="31"/>
       <c r="C153" s="31"/>
       <c r="D153" s="31"/>
       <c r="E153" s="31"/>
     </row>
-    <row r="154" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A154" s="31"/>
       <c r="B154" s="31"/>
       <c r="C154" s="31"/>
       <c r="D154" s="31"/>
       <c r="E154" s="31"/>
     </row>
-    <row r="155" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A155" s="31"/>
       <c r="B155" s="31"/>
       <c r="C155" s="31"/>
       <c r="D155" s="31"/>
       <c r="E155" s="31"/>
     </row>
-    <row r="156" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A156" s="31"/>
       <c r="B156" s="31"/>
       <c r="C156" s="31"/>
       <c r="D156" s="31"/>
       <c r="E156" s="31"/>
     </row>
-    <row r="157" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A157" s="31"/>
       <c r="B157" s="31"/>
       <c r="C157" s="31"/>
       <c r="D157" s="31"/>
       <c r="E157" s="31"/>
     </row>
-    <row r="158" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A158" s="31"/>
       <c r="B158" s="31"/>
       <c r="C158" s="31"/>
       <c r="D158" s="31"/>
       <c r="E158" s="31"/>
     </row>
-    <row r="159" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A159" s="31"/>
       <c r="B159" s="31"/>
       <c r="C159" s="31"/>
       <c r="D159" s="31"/>
       <c r="E159" s="31"/>
     </row>
-    <row r="160" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A160" s="31"/>
       <c r="B160" s="31"/>
       <c r="C160" s="31"/>
       <c r="D160" s="31"/>
       <c r="E160" s="31"/>
     </row>
-    <row r="161" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A161" s="31"/>
       <c r="B161" s="31"/>
       <c r="C161" s="31"/>
       <c r="D161" s="31"/>
       <c r="E161" s="31"/>
     </row>
-    <row r="162" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A162" s="31"/>
       <c r="B162" s="31"/>
       <c r="C162" s="31"/>
       <c r="D162" s="31"/>
       <c r="E162" s="31"/>
     </row>
-    <row r="163" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A163" s="31"/>
       <c r="B163" s="31"/>
       <c r="C163" s="31"/>
       <c r="D163" s="31"/>
       <c r="E163" s="31"/>
     </row>
-    <row r="164" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A164" s="31"/>
       <c r="B164" s="31"/>
       <c r="C164" s="31"/>
       <c r="D164" s="31"/>
       <c r="E164" s="31"/>
     </row>
-    <row r="165" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A165" s="31"/>
       <c r="B165" s="31"/>
       <c r="C165" s="31"/>
       <c r="D165" s="31"/>
       <c r="E165" s="31"/>
     </row>
-    <row r="166" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A166" s="31"/>
       <c r="B166" s="31"/>
       <c r="C166" s="31"/>
       <c r="D166" s="31"/>
       <c r="E166" s="31"/>
     </row>
-    <row r="167" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A167" s="31"/>
       <c r="B167" s="31"/>
       <c r="C167" s="31"/>
       <c r="D167" s="31"/>
       <c r="E167" s="31"/>
     </row>
-    <row r="168" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A168" s="31"/>
       <c r="B168" s="31"/>
       <c r="C168" s="31"/>
       <c r="D168" s="31"/>
       <c r="E168" s="31"/>
     </row>
-    <row r="169" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A169" s="31"/>
       <c r="B169" s="31"/>
       <c r="C169" s="31"/>
       <c r="D169" s="31"/>
       <c r="E169" s="31"/>
     </row>
-    <row r="170" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A170" s="31"/>
       <c r="B170" s="31"/>
       <c r="C170" s="31"/>
       <c r="D170" s="31"/>
       <c r="E170" s="31"/>
     </row>
-    <row r="171" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A171" s="31"/>
       <c r="B171" s="31"/>
       <c r="C171" s="31"/>
       <c r="D171" s="31"/>
       <c r="E171" s="31"/>
     </row>
-    <row r="172" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A172" s="31"/>
       <c r="B172" s="31"/>
       <c r="C172" s="31"/>
       <c r="D172" s="31"/>
       <c r="E172" s="31"/>
     </row>
-    <row r="173" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A173" s="31"/>
       <c r="B173" s="31"/>
       <c r="C173" s="31"/>
       <c r="D173" s="31"/>
       <c r="E173" s="31"/>
     </row>
-    <row r="174" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A174" s="31"/>
       <c r="B174" s="31"/>
       <c r="C174" s="31"/>
       <c r="D174" s="31"/>
       <c r="E174" s="31"/>
     </row>
-    <row r="175" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A175" s="31"/>
       <c r="B175" s="31"/>
       <c r="C175" s="31"/>
       <c r="D175" s="31"/>
       <c r="E175" s="31"/>
     </row>
-    <row r="176" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A176" s="31"/>
       <c r="B176" s="31"/>
       <c r="C176" s="31"/>
       <c r="D176" s="31"/>
       <c r="E176" s="31"/>
     </row>
-    <row r="177" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A177" s="31"/>
       <c r="B177" s="31"/>
       <c r="C177" s="31"/>
       <c r="D177" s="31"/>
       <c r="E177" s="31"/>
     </row>
-    <row r="178" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A178" s="31"/>
       <c r="B178" s="31"/>
       <c r="C178" s="31"/>
       <c r="D178" s="31"/>
       <c r="E178" s="31"/>
     </row>
-    <row r="179" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A179" s="31"/>
       <c r="B179" s="31"/>
       <c r="C179" s="31"/>
       <c r="D179" s="31"/>
       <c r="E179" s="31"/>
     </row>
-    <row r="180" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A180" s="31"/>
       <c r="B180" s="31"/>
       <c r="C180" s="31"/>
       <c r="D180" s="31"/>
       <c r="E180" s="31"/>
     </row>
-    <row r="181" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A181" s="31"/>
       <c r="B181" s="31"/>
       <c r="C181" s="31"/>
       <c r="D181" s="31"/>
       <c r="E181" s="31"/>
     </row>
-    <row r="182" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A182" s="31"/>
       <c r="B182" s="31"/>
       <c r="C182" s="31"/>
       <c r="D182" s="31"/>
       <c r="E182" s="31"/>
     </row>
-    <row r="183" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A183" s="31"/>
       <c r="B183" s="31"/>
       <c r="C183" s="31"/>
       <c r="D183" s="31"/>
       <c r="E183" s="31"/>
     </row>
-    <row r="184" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A184" s="31"/>
       <c r="B184" s="31"/>
       <c r="C184" s="31"/>
       <c r="D184" s="31"/>
       <c r="E184" s="31"/>
     </row>
-    <row r="185" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A185" s="31"/>
       <c r="B185" s="31"/>
       <c r="C185" s="31"/>
       <c r="D185" s="31"/>
       <c r="E185" s="31"/>
     </row>
-    <row r="186" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A186" s="31"/>
       <c r="B186" s="31"/>
       <c r="C186" s="31"/>
       <c r="D186" s="31"/>
       <c r="E186" s="31"/>
     </row>
-    <row r="187" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A187" s="31"/>
       <c r="B187" s="31"/>
       <c r="C187" s="31"/>
       <c r="D187" s="31"/>
       <c r="E187" s="31"/>
     </row>
-    <row r="188" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A188" s="31"/>
       <c r="B188" s="31"/>
       <c r="C188" s="31"/>
       <c r="D188" s="31"/>
       <c r="E188" s="31"/>
     </row>
-    <row r="189" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A189" s="31"/>
       <c r="B189" s="31"/>
       <c r="C189" s="31"/>
       <c r="D189" s="31"/>
       <c r="E189" s="31"/>
     </row>
-    <row r="190" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A190" s="31"/>
       <c r="B190" s="31"/>
       <c r="C190" s="31"/>
       <c r="D190" s="31"/>
       <c r="E190" s="31"/>
     </row>
-    <row r="191" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A191" s="31"/>
       <c r="B191" s="31"/>
       <c r="C191" s="31"/>
       <c r="D191" s="31"/>
       <c r="E191" s="31"/>
     </row>
-    <row r="192" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A192" s="31"/>
       <c r="B192" s="31"/>
       <c r="C192" s="31"/>
       <c r="D192" s="31"/>
       <c r="E192" s="31"/>
     </row>
-    <row r="193" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" ht="20" customHeight="1" ns3:dyDescent="0.2">
       <c r="A193" s="31"/>
       <c r="B193" s="31"/>
       <c r="C193" s="31"/>

</xml_diff>